<commit_message>
Harden Phase 7 reporting cycle readiness
</commit_message>
<xml_diff>
--- a/05_reporting_controls/data_quality/data_quality_framework.xlsx
+++ b/05_reporting_controls/data_quality/data_quality_framework.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQ Overview" sheetId="1" r:id="R6bf42e346e5a45bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules Matrix" sheetId="2" r:id="Re6f356f7b4534bac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observed Findings" sheetId="3" r:id="R078af1f3cfa447b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="4" r:id="Reb9ea024b84c478e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controlled Tests" sheetId="5" r:id="R9b9da4a0bc5a4b45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Inventory" sheetId="6" r:id="Rc9d9f02337c045bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQ Overview" sheetId="1" r:id="R4c4acf21103c4b5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules Matrix" sheetId="2" r:id="Re731d2e2202242a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observed Findings" sheetId="3" r:id="Rcb659bd393e54ff3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="4" r:id="R0d63e32c2e7e45a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controlled Tests" sheetId="5" r:id="R75ef358e1ddc41fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Inventory" sheetId="6" r:id="R1808f2baf29e448f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,7 +18,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="6">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -52,8 +52,14 @@
       <x:color rgb="FF7F6000"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -88,6 +94,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -206,7 +227,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="62">
+  <x:cellXfs count="68">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -339,6 +360,14 @@
     <x:xf numFmtId="0" fontId="5" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -350,7 +379,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -360,7 +389,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -371,7 +400,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -382,7 +411,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -393,7 +422,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -404,7 +433,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -414,7 +443,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DQRulesMatrix" displayName="DQRulesMatrix" ref="A5:M44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DQRulesMatrix" displayName="DQRulesMatrix" ref="A5:M47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Rule ID"/>
     <x:tableColumn id="2" name="Dataset"/>
@@ -449,7 +478,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ControlledTests" displayName="ControlledTests" ref="A5:E17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ControlledTests" displayName="ControlledTests" ref="A5:E19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Control area"/>
@@ -693,7 +722,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Observed NHS source findings are separated from controlled pipeline tests. Clean reporting outputs contain Accepted records only.</x:v>
+        <x:v>Observed source findings are separated from controlled tests and approved mapping/schema decisions. Clean reporting outputs require Accepted status and the approved London cohort.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -787,6 +816,16 @@
       <x:c r="G8" s="10"/>
       <x:c r="H8" s="10"/>
     </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="63" t="str">
+        <x:v>Baseline source profile before reference and schema approvals</x:v>
+      </x:c>
+      <x:c r="B9" s="63"/>
+      <x:c r="C9" s="63"/>
+      <x:c r="D9" s="63"/>
+      <x:c r="E9" s="63"/>
+      <x:c r="F9" s="63"/>
+    </x:row>
     <x:row r="10" ht="34" customHeight="1">
       <x:c r="A10" s="22" t="str">
         <x:v>Dataset</x:v>
@@ -884,7 +923,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="53" t="str">
-        <x:v>Do not publish when a Critical rule is unresolved, an unclassified difference is non-zero, or rejected/review totals are unexplained. Organisation names are descriptive fields only; OrganisationCode + ReportingMonth is the shared comparison key.</x:v>
+        <x:v>Do not publish when a Critical rule is unresolved, an unclassified difference is non-zero, or quality/scope differences are unexplained. Operational outputs use the controlled 148-code reference and the 20-provider London cohort.</x:v>
       </x:c>
       <x:c r="B16" s="54"/>
       <x:c r="C16" s="54"/>
@@ -931,6 +970,7 @@
     <x:mergeCell ref="A4:H4"/>
     <x:mergeCell ref="A15:H15"/>
     <x:mergeCell ref="A16:H19"/>
+    <x:mergeCell ref="A9:F9"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1946,19 +1986,19 @@
         <x:v>All source fields</x:v>
       </x:c>
       <x:c r="E28" s="31" t="str">
-        <x:v>Unexpected columns must be identified and excluded from the canonical model.</x:v>
+        <x:v>Unexpected columns containing data require review; approved blank trailing artifacts are projected out.</x:v>
       </x:c>
       <x:c r="F28" s="31" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G28" s="31" t="str">
-        <x:v>No unexpected columns.</x:v>
+        <x:v>No unexpected column contains row data unless explicitly approved.</x:v>
       </x:c>
       <x:c r="H28" s="31" t="str">
         <x:v>Unexpected header names and SourceFile.</x:v>
       </x:c>
       <x:c r="I28" s="31" t="str">
-        <x:v>Review Required</x:v>
+        <x:v>Review Required or approved warning</x:v>
       </x:c>
       <x:c r="J28" s="31" t="str">
         <x:v>Unreviewed fields may signal an upstream layout change.</x:v>
@@ -1970,7 +2010,7 @@
         <x:v>Observed source issue</x:v>
       </x:c>
       <x:c r="M28" s="31" t="str">
-        <x:v>2024-09 contains five blank headers and one header named a.</x:v>
+        <x:v>2024-09 has six extra headers with no row data; approved canonical projection.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="76" customHeight="1">
@@ -2397,7 +2437,7 @@
         <x:v>OrganisationCode</x:v>
       </x:c>
       <x:c r="E39" s="31" t="str">
-        <x:v>Codes must match the approved DimOrganisation reference once that reference is built.</x:v>
+        <x:v>Codes must match the controlled stable DimOrganisation reference.</x:v>
       </x:c>
       <x:c r="F39" s="31" t="str">
         <x:v>High</x:v>
@@ -2421,7 +2461,7 @@
         <x:v>Controlled pipeline test</x:v>
       </x:c>
       <x:c r="M39" s="31" t="str">
-        <x:v>Reference dimension is not yet populated; rule is intentionally pending.</x:v>
+        <x:v>Reference populated with 148 stable codes; 20 London providers are reportable.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="76" customHeight="1">
@@ -2561,13 +2601,13 @@
         <x:v>SourceFile + LoadTimestamp</x:v>
       </x:c>
       <x:c r="E43" s="31" t="str">
-        <x:v>Every refresh must retain source lineage and a fixed UTC timestamp.</x:v>
+        <x:v>Every refresh must retain source, file-version, load, status and validation lineage.</x:v>
       </x:c>
       <x:c r="F43" s="31" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="G43" s="31" t="str">
-        <x:v>All classified rows have the six mandatory provenance fields.</x:v>
+        <x:v>All classified rows have the ten mandatory provenance fields.</x:v>
       </x:c>
       <x:c r="H43" s="31" t="str">
         <x:v>Rows missing provenance.</x:v>
@@ -2579,13 +2619,13 @@
         <x:v>Issues cannot be traced to the source file or refresh.</x:v>
       </x:c>
       <x:c r="K43" s="31" t="str">
-        <x:v>Add provenance in transform functions; not-null checks in control query.</x:v>
+        <x:v>Add file metadata in staging and status lineage in classified queries.</x:v>
       </x:c>
       <x:c r="L43" s="31" t="str">
         <x:v>Observed source check</x:v>
       </x:c>
       <x:c r="M43" s="31" t="str">
-        <x:v>Implemented in all three transformations.</x:v>
+        <x:v>Implemented across the three staging and classification pipelines.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="76" customHeight="1">
@@ -2602,13 +2642,13 @@
         <x:v>Source file manifest and previous refresh</x:v>
       </x:c>
       <x:c r="E44" s="31" t="str">
-        <x:v>File hash, row count and measure totals should be compared with the previous refresh.</x:v>
+        <x:v>Active, duplicate and revised files must be identified for each dataset-month.</x:v>
       </x:c>
       <x:c r="F44" s="31" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="G44" s="31" t="str">
-        <x:v>Changes are either zero or documented as a revision/new reporting period.</x:v>
+        <x:v>Exactly one Active file exists per valid dataset-month and older versions are classified.</x:v>
       </x:c>
       <x:c r="H44" s="31" t="str">
         <x:v>Changed file hash, rows, totals and commentary reason.</x:v>
@@ -2620,13 +2660,136 @@
         <x:v>Silent republication can rewrite reported history.</x:v>
       </x:c>
       <x:c r="K44" s="31" t="str">
-        <x:v>Persist refresh summary and compare to prior snapshot.</x:v>
+        <x:v>fnGetSourceFiles and qrySourceFileRegister; archive hashes remain external control evidence.</x:v>
       </x:c>
       <x:c r="L44" s="31" t="str">
         <x:v>Controlled pipeline test</x:v>
       </x:c>
       <x:c r="M44" s="31" t="str">
-        <x:v>Workforce extraction manifest exists; full refresh history begins after first Excel refresh.</x:v>
+        <x:v>Implemented; cycle history begins with the first Phase 7 refresh.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A45" s="10" t="str">
+        <x:v>DQ-X-004</x:v>
+      </x:c>
+      <x:c r="B45" s="10" t="str">
+        <x:v>All datasets</x:v>
+      </x:c>
+      <x:c r="C45" s="10" t="str">
+        <x:v>Revision control</x:v>
+      </x:c>
+      <x:c r="D45" s="10" t="str">
+        <x:v>SourceFile + FileReportingMonth</x:v>
+      </x:c>
+      <x:c r="E45" s="10" t="str">
+        <x:v>Only the latest modified file for a dataset-month is transformed.</x:v>
+      </x:c>
+      <x:c r="F45" s="10" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G45" s="10" t="str">
+        <x:v>FileVersionRank 1 is Active; all older files have an explained disposition.</x:v>
+      </x:c>
+      <x:c r="H45" s="10" t="str">
+        <x:v>File register row with version rank and reason.</x:v>
+      </x:c>
+      <x:c r="I45" s="10" t="str">
+        <x:v>Supersede older version</x:v>
+      </x:c>
+      <x:c r="J45" s="10" t="str">
+        <x:v>Loading two versions duplicates or rewrites reported results.</x:v>
+      </x:c>
+      <x:c r="K45" s="10" t="str">
+        <x:v>fnGetSourceFiles groups and ranks source files before transformation.</x:v>
+      </x:c>
+      <x:c r="L45" s="10" t="str">
+        <x:v>Controlled pipeline test</x:v>
+      </x:c>
+      <x:c r="M45" s="10" t="str">
+        <x:v>No duplicate local month files in the baseline folders.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A46" s="10" t="str">
+        <x:v>DQ-X-005</x:v>
+      </x:c>
+      <x:c r="B46" s="10" t="str">
+        <x:v>All datasets</x:v>
+      </x:c>
+      <x:c r="C46" s="10" t="str">
+        <x:v>Reporting scope</x:v>
+      </x:c>
+      <x:c r="D46" s="10" t="str">
+        <x:v>InclusionFlag</x:v>
+      </x:c>
+      <x:c r="E46" s="10" t="str">
+        <x:v>Only approved London-cohort organisations reach clean outputs.</x:v>
+      </x:c>
+      <x:c r="F46" s="10" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="G46" s="10" t="str">
+        <x:v>Every clean row has InclusionFlag = true.</x:v>
+      </x:c>
+      <x:c r="H46" s="10" t="str">
+        <x:v>Accepted out-of-scope row and organisation reference evidence.</x:v>
+      </x:c>
+      <x:c r="I46" s="10" t="str">
+        <x:v>Scope exclusion</x:v>
+      </x:c>
+      <x:c r="J46" s="10" t="str">
+        <x:v>Mixing the national universe with the management cohort changes totals and coverage.</x:v>
+      </x:c>
+      <x:c r="K46" s="10" t="str">
+        <x:v>Join dimOrganisation; filter clean queries on Accepted and InclusionFlag.</x:v>
+      </x:c>
+      <x:c r="L46" s="10" t="str">
+        <x:v>Control rule</x:v>
+      </x:c>
+      <x:c r="M46" s="10" t="str">
+        <x:v>20 London providers selected from the 148-code stable intersection.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A47" s="10" t="str">
+        <x:v>DQ-REC-005</x:v>
+      </x:c>
+      <x:c r="B47" s="10" t="str">
+        <x:v>All datasets</x:v>
+      </x:c>
+      <x:c r="C47" s="10" t="str">
+        <x:v>Scope reconciliation</x:v>
+      </x:c>
+      <x:c r="D47" s="10" t="str">
+        <x:v>AcceptedValue + ReportableValue</x:v>
+      </x:c>
+      <x:c r="E47" s="10" t="str">
+        <x:v>Accepted totals must reconcile to reportable totals plus documented scope exclusions.</x:v>
+      </x:c>
+      <x:c r="F47" s="10" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G47" s="10" t="str">
+        <x:v>AcceptedValue - ReportableValue equals the controlled scope exclusion.</x:v>
+      </x:c>
+      <x:c r="H47" s="10" t="str">
+        <x:v>Metric, accepted total, reportable total and difference reason.</x:v>
+      </x:c>
+      <x:c r="I47" s="10" t="str">
+        <x:v>Publication gate</x:v>
+      </x:c>
+      <x:c r="J47" s="10" t="str">
+        <x:v>A scope change can be mistaken for a data-quality loss or performance movement.</x:v>
+      </x:c>
+      <x:c r="K47" s="10" t="str">
+        <x:v>qryDataQualityReconciliation exposes raw, accepted and reportable values.</x:v>
+      </x:c>
+      <x:c r="L47" s="10" t="str">
+        <x:v>Control rule</x:v>
+      </x:c>
+      <x:c r="M47" s="10" t="str">
+        <x:v>Implemented for row counts and additive measures.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2643,7 +2806,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2aab0d62ca2d418b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12c1e6ecb5764627"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2874,10 +3037,10 @@
         <x:v>RAX, RW1, RWD, RRE; 48 affected rows</x:v>
       </x:c>
       <x:c r="E14" s="31" t="str">
-        <x:v>Review Required</x:v>
+        <x:v>Approved mapping</x:v>
       </x:c>
       <x:c r="F14" s="31" t="str">
-        <x:v>Likely renames or reorganisations; confirm in organisation mapping.</x:v>
+        <x:v>Alias histories are documented in dim_organisation.csv; names remain display fields only.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="60" customHeight="1">
@@ -2914,10 +3077,10 @@
         <x:v>Five blank headers and one header named a</x:v>
       </x:c>
       <x:c r="E16" s="31" t="str">
-        <x:v>Review Required</x:v>
+        <x:v>Approved warning</x:v>
       </x:c>
       <x:c r="F16" s="31" t="str">
-        <x:v>Canonical 22 columns remain present; extras are ignored explicitly.</x:v>
+        <x:v>Extra columns contain no row data; the canonical 22 fields are selected by name.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="60" customHeight="1">
@@ -2994,10 +3157,10 @@
         <x:v>RAX, RW1, RWD</x:v>
       </x:c>
       <x:c r="E20" s="31" t="str">
-        <x:v>Review Required</x:v>
+        <x:v>Approved mapping</x:v>
       </x:c>
       <x:c r="F20" s="31" t="str">
-        <x:v>Likely the same renames seen in absence files.</x:v>
+        <x:v>Alias histories are documented in dim_organisation.csv.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3012,7 +3175,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36158ff22c7a4bbf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4931706e4e064116"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3027,8 +3190,9 @@
     <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="66" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="31" customHeight="1">
@@ -3045,7 +3209,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Current source-profile row counts and the required reconciliation controls for every Excel refresh.</x:v>
+        <x:v>Baseline source-profile counts are shown first. Operational refreshes must also reconcile accepted totals to the approved London reportable cohort.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -3063,15 +3227,18 @@
         <x:v>Raw rows</x:v>
       </x:c>
       <x:c r="C5" s="23" t="str">
-        <x:v>Accepted</x:v>
+        <x:v>Baseline Accepted</x:v>
       </x:c>
       <x:c r="D5" s="23" t="str">
-        <x:v>Review Required</x:v>
+        <x:v>Baseline Review</x:v>
       </x:c>
       <x:c r="E5" s="23" t="str">
-        <x:v>Rejected</x:v>
+        <x:v>Baseline Rejected</x:v>
       </x:c>
       <x:c r="F5" s="24" t="str">
+        <x:v>Reportable cohort</x:v>
+      </x:c>
+      <x:c r="G5" s="65" t="str">
         <x:v>Difference</x:v>
       </x:c>
     </x:row>
@@ -3092,7 +3259,9 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F6" s="32" t="n">
-        <x:f>B6-SUM(C6:E6)</x:f>
+        <x:v>11352</x:v>
+      </x:c>
+      <x:c r="G6" s="66" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3113,7 +3282,9 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="33" t="n">
-        <x:f>B7-SUM(C7:E7)</x:f>
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="G7" s="66" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3134,11 +3305,13 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="F8" s="33" t="n">
-        <x:f>B8-SUM(C8:E8)</x:f>
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="G8" s="66" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="34" customHeight="1">
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="22" t="str">
         <x:v>Dataset</x:v>
       </x:c>
@@ -3152,19 +3325,22 @@
         <x:v>Accepted total</x:v>
       </x:c>
       <x:c r="E11" s="23" t="str">
+        <x:v>Reportable total</x:v>
+      </x:c>
+      <x:c r="F11" s="23" t="str">
         <x:v>Review total</x:v>
       </x:c>
-      <x:c r="F11" s="23" t="str">
+      <x:c r="G11" s="23" t="str">
         <x:v>Rejected total</x:v>
       </x:c>
-      <x:c r="G11" s="23" t="str">
+      <x:c r="H11" s="24" t="str">
         <x:v>Difference</x:v>
       </x:c>
-      <x:c r="H11" s="24" t="str">
+      <x:c r="I11" s="67" t="str">
         <x:v>Difference reason</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="52" customHeight="1">
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="30" t="str">
         <x:v>Workforce</x:v>
       </x:c>
@@ -3184,13 +3360,16 @@
         <x:v>Power Query refresh</x:v>
       </x:c>
       <x:c r="G12" s="30" t="str">
+        <x:v>Power Query refresh</x:v>
+      </x:c>
+      <x:c r="H12" s="30" t="str">
         <x:v>Calculated by qryDataQualityReconciliation</x:v>
       </x:c>
-      <x:c r="H12" s="30" t="str">
-        <x:v>Status totals must explain the difference; percentages are never summed.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="52" customHeight="1">
+      <x:c r="I12" s="10" t="str">
+        <x:v>Quality and scope differences are reported separately.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A13" s="31" t="str">
         <x:v>Workforce</x:v>
       </x:c>
@@ -3210,13 +3389,16 @@
         <x:v>Power Query refresh</x:v>
       </x:c>
       <x:c r="G13" s="31" t="str">
+        <x:v>Power Query refresh</x:v>
+      </x:c>
+      <x:c r="H13" s="31" t="str">
         <x:v>Calculated by qryDataQualityReconciliation</x:v>
       </x:c>
-      <x:c r="H13" s="31" t="str">
+      <x:c r="I13" s="10" t="str">
         <x:v>Use the intended total/member rule to prevent double counting.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="52" customHeight="1">
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="31" t="str">
         <x:v>Absence</x:v>
       </x:c>
@@ -3236,13 +3418,16 @@
         <x:v>Power Query refresh</x:v>
       </x:c>
       <x:c r="G14" s="31" t="str">
+        <x:v>Power Query refresh</x:v>
+      </x:c>
+      <x:c r="H14" s="31" t="str">
         <x:v>Calculated by qryDataQualityReconciliation</x:v>
       </x:c>
-      <x:c r="H14" s="31" t="str">
+      <x:c r="I14" s="10" t="str">
         <x:v>Additive measure reconciliation.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="52" customHeight="1">
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="31" t="str">
         <x:v>Absence</x:v>
       </x:c>
@@ -3262,13 +3447,16 @@
         <x:v>Power Query refresh</x:v>
       </x:c>
       <x:c r="G15" s="31" t="str">
+        <x:v>Power Query refresh</x:v>
+      </x:c>
+      <x:c r="H15" s="31" t="str">
         <x:v>Calculated by qryDataQualityReconciliation</x:v>
       </x:c>
-      <x:c r="H15" s="31" t="str">
+      <x:c r="I15" s="10" t="str">
         <x:v>Additive measure reconciliation.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="52" customHeight="1">
+    <x:row r="16" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A16" s="31" t="str">
         <x:v>A&amp;E Activity</x:v>
       </x:c>
@@ -3288,13 +3476,16 @@
         <x:v>Power Query refresh</x:v>
       </x:c>
       <x:c r="G16" s="31" t="str">
+        <x:v>Power Query refresh</x:v>
+      </x:c>
+      <x:c r="H16" s="31" t="str">
         <x:v>Calculated by qryDataQualityReconciliation</x:v>
       </x:c>
-      <x:c r="H16" s="31" t="str">
+      <x:c r="I16" s="10" t="str">
         <x:v>Type 1 + Type 2 + Other; booked subsets are not added again.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="52" customHeight="1">
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="31" t="str">
         <x:v>A&amp;E Activity</x:v>
       </x:c>
@@ -3314,13 +3505,16 @@
         <x:v>Power Query refresh</x:v>
       </x:c>
       <x:c r="G17" s="31" t="str">
+        <x:v>Power Query refresh</x:v>
+      </x:c>
+      <x:c r="H17" s="31" t="str">
         <x:v>Calculated by qryDataQualityReconciliation</x:v>
       </x:c>
-      <x:c r="H17" s="31" t="str">
+      <x:c r="I17" s="10" t="str">
         <x:v>Corresponding non-booked headline fields only.</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="52" customHeight="1">
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="31" t="str">
         <x:v>A&amp;E Activity</x:v>
       </x:c>
@@ -3340,9 +3534,12 @@
         <x:v>Power Query refresh</x:v>
       </x:c>
       <x:c r="G18" s="31" t="str">
+        <x:v>Power Query refresh</x:v>
+      </x:c>
+      <x:c r="H18" s="31" t="str">
         <x:v>Calculated by qryDataQualityReconciliation</x:v>
       </x:c>
-      <x:c r="H18" s="31" t="str">
+      <x:c r="I18" s="10" t="str">
         <x:v>All four admission fields are additive.</x:v>
       </x:c>
     </x:row>
@@ -3585,7 +3782,7 @@
         <x:v>The record becomes Review Required in the unmatched-organisation output.</x:v>
       </x:c>
       <x:c r="E16" s="31" t="str">
-        <x:v>Pending until DimOrganisation is populated</x:v>
+        <x:v>Reference populated with 148 stable codes; unmatched-code behaviour remains a controlled test.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="66" customHeight="1">
@@ -3603,6 +3800,40 @@
       </x:c>
       <x:c r="E17" s="31" t="str">
         <x:v>Not observed; pipeline control</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A18" s="10" t="str">
+        <x:v>TC-013</x:v>
+      </x:c>
+      <x:c r="B18" s="10" t="str">
+        <x:v>Revision control</x:v>
+      </x:c>
+      <x:c r="C18" s="10" t="str">
+        <x:v>Add an identical renamed copy and a non-identical revised copy for one month.</x:v>
+      </x:c>
+      <x:c r="D18" s="10" t="str">
+        <x:v>The latest file is Active; older files are classified duplicate or revised and are not transformed.</x:v>
+      </x:c>
+      <x:c r="E18" s="10" t="str">
+        <x:v>Phase 7 controlled test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A19" s="10" t="str">
+        <x:v>TC-014</x:v>
+      </x:c>
+      <x:c r="B19" s="10" t="str">
+        <x:v>Reporting scope</x:v>
+      </x:c>
+      <x:c r="C19" s="10" t="str">
+        <x:v>Set InclusionFlag to false for one otherwise Accepted provider.</x:v>
+      </x:c>
+      <x:c r="D19" s="10" t="str">
+        <x:v>The record remains Accepted in quality status but is excluded from reportable clean output and scope difference increases.</x:v>
+      </x:c>
+      <x:c r="E19" s="10" t="str">
+        <x:v>Phase 7 controlled test</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3612,7 +3843,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6290df39248245c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R535694ce94b34611"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4452,7 +4683,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3354552f265742a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3fa0c18436b49cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>